<commit_message>
Updated Cordulegaster helladica sprawler -> burrower
</commit_message>
<xml_diff>
--- a/data/OdonTraits_Europe.xlsx
+++ b/data/OdonTraits_Europe.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="12460"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="12460" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="taxonomic" sheetId="2" r:id="rId1"/>
@@ -15375,7 +15375,7 @@
         <v>536</v>
       </c>
       <c r="O47" s="10" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
     </row>
     <row r="48" spans="1:15" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
updated habitat for Ischnura hastata (eutrophic -> oligotrophic) and Orthetrum ransonnetii (percher -> flier)
</commit_message>
<xml_diff>
--- a/data/OdonTraits_Europe.xlsx
+++ b/data/OdonTraits_Europe.xlsx
@@ -16463,8 +16463,8 @@
       <c r="A71" t="s">
         <v>170</v>
       </c>
-      <c r="B71" s="3" t="s">
-        <v>12</v>
+      <c r="B71" s="1" t="s">
+        <v>7</v>
       </c>
       <c r="C71" s="12" t="s">
         <v>527</v>
@@ -18018,7 +18018,7 @@
         <v>588</v>
       </c>
       <c r="C104" s="12" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
       <c r="D104" t="s">
         <v>562</v>

</xml_diff>